<commit_message>
non convexity solved: local opt neighborhood search added to find the truning points, then searching for local opts, and then reporting global opt. both cvar and var. for var may not be necessary.
</commit_message>
<xml_diff>
--- a/reports/~opt_cvar_report.xlsx
+++ b/reports/~opt_cvar_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iesegnet-my.sharepoint.com/personal/s_rostami_ieseg_fr/Documents/Research/Papers/2020-eNPV_Contract/NPV Risk Contract - Python/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{5C601A5B-4CFB-4AB4-BB1A-AE32044B64AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D0CC100-F920-4AD8-86F0-21EE1551E218}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{5C601A5B-4CFB-4AB4-BB1A-AE32044B64AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB51DF4-061B-48C7-B0EF-6B277CD5C137}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{95B63630-DBFE-4F93-86A4-4F5FA770A2A7}"/>
   </bookViews>
@@ -636,6 +636,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -967,7 +971,9 @@
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">

</xml_diff>